<commit_message>
Agenda workbook: one row per section
</commit_message>
<xml_diff>
--- a/AI_Steerco_Kickoff_Agenda.xlsx
+++ b/AI_Steerco_Kickoff_Agenda.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ask tracker" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Agenda'!$A$5:$M$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Agenda'!$A$5:$M$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'People and groups'!$A$3:$D$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -519,9 +519,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Planned start time</t>
+          <t>Start time</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
@@ -564,11 +564,11 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Total planned (minutes)</t>
+          <t>Total min</t>
         </is>
       </c>
       <c r="C3" s="2">
-        <f>SUM(D6:D41)</f>
+        <f>SUM(D6:D18)</f>
         <v/>
       </c>
       <c r="D3" s="4">
@@ -643,7 +643,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="33.75" customHeight="1">
       <c r="A6" s="6" t="n">
         <v>1</v>
       </c>
@@ -670,7 +670,7 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>People join and the tech settles. If we start on time, use it to begin the opening early.</t>
+          <t>• People join and the tech settles. If we start on time, use it to begin early. (10 min)</t>
         </is>
       </c>
       <c r="H6" s="9" t="inlineStr">
@@ -696,7 +696,7 @@
       </c>
       <c r="M6" s="9" t="inlineStr"/>
     </row>
-    <row r="7">
+    <row r="7" ht="33.75" customHeight="1">
       <c r="A7" s="10" t="n">
         <v>2</v>
       </c>
@@ -723,9 +723,7 @@
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>• Why we are kicking off
-• What we are covering today (and that it is not everything we will ever cover)
-• How the open call and open forum work</t>
+          <t>• Why we are kicking off, what we are covering (not everything we will ever cover), and how the open call and open forum work (5 min)</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
@@ -751,11 +749,11 @@
       </c>
       <c r="M7" s="13" t="inlineStr">
         <is>
-          <t>Proposed. You did not list an opening, so change or cut as you like.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+          <t>Proposed. You did not list an opening, so change or cut it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="303.75" customHeight="1">
       <c r="A8" s="10" t="n">
         <v>3</v>
       </c>
@@ -768,7 +766,7 @@
         <v/>
       </c>
       <c r="D8" s="10" t="n">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
@@ -777,45 +775,60 @@
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>The journey (one slide)</t>
+          <t>Dan Knauf: journey, fireside chat, click-downs</t>
         </is>
       </c>
       <c r="G8" s="13" t="inlineStr">
         <is>
-          <t>• Where we stood with AI before Dan
-• Dan joins (his photo)
-• What has happened since, up to now
-• The horizon: where we are going</t>
+          <t>• The journey, one slide: where we stood before Dan, Dan joins (his photo), what has happened since, and the horizon | Dan Knauf (4 min)
+• Fireside chat | Rachel Harris, Dan Knauf (12 min)
+      Warm-up
+      - What did you think AI was doing here when you walked in, and what surprised you most?
+      - What has gone better than you expected, and what has gone worse?
+      The journey
+      - If AI could take one task off everyone's plate tomorrow, what should it be?
+      - What worries you most about AI here, and what gets you most excited?
+      Looking ahead
+      - What do you want this room to do in the next 90 days?
+      - Rapid fire: favorite tool right now, one thing you would retire, one prediction.
+• Click-down: asking for more budget, and what that means for the teams | Dan Knauf (6 min)
+• Click-down: Multiplayer | Dan Knauf (3 min)
+• Click-down: Vercel | Dan Knauf (3 min)
+• Click-down: Local LLMs | Dan Knauf (2 min)</t>
         </is>
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>Dan Knauf</t>
+          <t>Dan Knauf, Rachel Harris</t>
         </is>
       </c>
       <c r="I8" s="13" t="inlineStr">
         <is>
-          <t>CTO</t>
+          <t>CTO; Ops</t>
         </is>
       </c>
       <c r="J8" s="13" t="inlineStr">
         <is>
-          <t>One slide</t>
+          <t>Slide + fireside + click-downs</t>
         </is>
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>One slide. Dan sends a few milestones; Rachel can draft it.</t>
+          <t>One journey slide (Dan sends milestones; Rachel can draft). Short prompt slides for the four click-downs. None for the fireside.</t>
         </is>
       </c>
       <c r="L8" s="13" t="inlineStr">
         <is>
-          <t>Must keep</t>
-        </is>
-      </c>
-      <c r="M8" s="13" t="inlineStr"/>
-    </row>
-    <row r="9">
+          <t>Shorten fireside to 8; Vercel and Local LLMs can go in writing</t>
+        </is>
+      </c>
+      <c r="M8" s="13" t="inlineStr">
+        <is>
+          <t>Assumes Rachel hosts the fireside. You have not said what to cover on Multiplayer, Vercel and Local LLMs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="114.75" customHeight="1">
       <c r="A9" s="10" t="n">
         <v>4</v>
       </c>
@@ -828,60 +841,57 @@
         <v/>
       </c>
       <c r="D9" s="10" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>1. Dan Knauf</t>
+          <t>2. Risk Review and priorities</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>Fireside chat</t>
+          <t>Risk Review and priorities</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>• Most impressive thing you have seen someone here build with AI?
-• What did we try that flopped, and what did it teach us?
-• What do people get wrong about what you do?
-• Which team should everyone borrow ideas from?
-• If AI could take one task off everyone's plate, what?
-• What worries you most, and what excites you most?</t>
+          <t>• What the team is doing to speed up reviews: update on the meeting Dan had with the Risk team, Shawn Street and Trisha (4 min)
+• Ask 1: start working on priorities we can surface in these calls, so we can prioritize requests and guide teams to ours (lots of things come in) (5 min)
+• Ask 2: how we show up when entering requests. Example of a really good request; if we want things to move fast, the business side must respond fast too (6 min)</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Rachel Harris, Dan Knauf</t>
+          <t>Dan Knauf, Trisha Scott</t>
         </is>
       </c>
       <c r="I9" s="13" t="inlineStr">
         <is>
-          <t>Ops; CTO</t>
+          <t>CTO; Legal</t>
         </is>
       </c>
       <c r="J9" s="13" t="inlineStr">
         <is>
-          <t>Fireside</t>
+          <t>Update, asks, discussion</t>
         </is>
       </c>
       <c r="K9" s="13" t="inlineStr">
         <is>
-          <t>None. Dan reviews the questions.</t>
+          <t>A few bullets on the meetings. One real example of a strong request.</t>
         </is>
       </c>
       <c r="L9" s="13" t="inlineStr">
         <is>
-          <t>Shorten to 6 min</t>
+          <t>Must keep</t>
         </is>
       </c>
       <c r="M9" s="13" t="inlineStr">
         <is>
-          <t>Assumes Rachel hosts. Change if someone else does.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
+          <t>Shawn Street is not on the roster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="47.25" customHeight="1">
       <c r="A10" s="10" t="n">
         <v>5</v>
       </c>
@@ -894,51 +904,52 @@
         <v/>
       </c>
       <c r="D10" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>1. Dan Knauf</t>
+          <t>3. AI market moves</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>Click-down: asking for more budget</t>
+          <t>AI market moves</t>
         </is>
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>What it would mean for the teams.</t>
+          <t>• Quick pulse on what competitors are doing specifically with AI (4 min)
+• Discussion: ideas, things we could learn (4 min)</t>
         </is>
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>Dan Knauf</t>
+          <t>Katherine Jones-Siemsen</t>
         </is>
       </c>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>CTO</t>
+          <t>Strategy</t>
         </is>
       </c>
       <c r="J10" s="13" t="inlineStr">
         <is>
-          <t>Click-down</t>
+          <t>Update + discussion</t>
         </is>
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>A short prompt slide.</t>
+          <t>A few slides or a one-page summary.</t>
         </is>
       </c>
       <c r="L10" s="13" t="inlineStr">
         <is>
-          <t>Must keep</t>
+          <t>Shorten to 5 min</t>
         </is>
       </c>
       <c r="M10" s="13" t="inlineStr"/>
     </row>
-    <row r="11">
+    <row r="11" ht="101.25" customHeight="1">
       <c r="A11" s="10" t="n">
         <v>6</v>
       </c>
@@ -951,116 +962,110 @@
         <v/>
       </c>
       <c r="D11" s="10" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>1. Dan Knauf</t>
+          <t>4. Best practice hub</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>Click-down: Multiplayer</t>
+          <t>Best practice hub</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>Dan to speak to it.</t>
+          <t>• Vision: one place for skills, plugins, connectors and shared context, tagged by role and craft (5 min)
+      We do not have the hub yet. Create Hub has started it and is our framework to get kicked off (ties to Design System Agentification)
+• Open discussion: where we see it going, and the value across the org (7 min)</t>
         </is>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>Dan Knauf</t>
+          <t>Dan Knauf, Dave Brabec</t>
         </is>
       </c>
       <c r="I11" s="13" t="inlineStr">
         <is>
-          <t>CTO</t>
+          <t>CTO; Ops</t>
         </is>
       </c>
       <c r="J11" s="13" t="inlineStr">
         <is>
-          <t>Click-down</t>
+          <t>Slides + discussion</t>
         </is>
       </c>
       <c r="K11" s="13" t="inlineStr">
         <is>
-          <t>A short prompt slide.</t>
+          <t>A few slides.</t>
         </is>
       </c>
       <c r="L11" s="13" t="inlineStr">
         <is>
-          <t>Shorten or send in writing</t>
+          <t>Must keep</t>
         </is>
       </c>
       <c r="M11" s="13" t="inlineStr">
         <is>
-          <t>You have not said what to cover on this one.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="n">
+          <t>Line up with Dave Calleja, who covers Design System Agentification in the DBT section.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="33.75" customHeight="1">
+      <c r="A12" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="7">
         <f>C11</f>
         <v/>
       </c>
-      <c r="C12" s="11">
+      <c r="C12" s="7">
         <f>B12+D12/1440</f>
         <v/>
       </c>
-      <c r="D12" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E12" s="12" t="inlineStr">
-        <is>
-          <t>1. Dan Knauf</t>
-        </is>
-      </c>
-      <c r="F12" s="12" t="inlineStr">
-        <is>
-          <t>Click-down: Vercel</t>
-        </is>
-      </c>
-      <c r="G12" s="13" t="inlineStr">
-        <is>
-          <t>Dan to speak to it.</t>
-        </is>
-      </c>
-      <c r="H12" s="13" t="inlineStr">
-        <is>
-          <t>Dan Knauf</t>
-        </is>
-      </c>
-      <c r="I12" s="13" t="inlineStr">
-        <is>
-          <t>CTO</t>
-        </is>
-      </c>
-      <c r="J12" s="13" t="inlineStr">
-        <is>
-          <t>Click-down</t>
-        </is>
-      </c>
-      <c r="K12" s="13" t="inlineStr">
-        <is>
-          <t>A short prompt slide.</t>
-        </is>
-      </c>
-      <c r="L12" s="13" t="inlineStr">
-        <is>
-          <t>Shorten or send in writing</t>
-        </is>
-      </c>
-      <c r="M12" s="13" t="inlineStr">
-        <is>
-          <t>You have not said what to cover on this one.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
+      <c r="D12" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Break</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Break</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>• Stretch and refill. If we are running late, shorten to 5 minutes. (10 min)</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Rachel Harris</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>Ops</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>Break</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr"/>
+      <c r="L12" s="9" t="inlineStr">
+        <is>
+          <t>Shorten to 5 min</t>
+        </is>
+      </c>
+      <c r="M12" s="9" t="inlineStr"/>
+    </row>
+    <row r="13" ht="114.75" customHeight="1">
       <c r="A13" s="10" t="n">
         <v>8</v>
       </c>
@@ -1073,55 +1078,59 @@
         <v/>
       </c>
       <c r="D13" s="10" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>1. Dan Knauf</t>
+          <t>5. DBT</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>Click-down: Local LLMs</t>
+          <t>DBT</t>
         </is>
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>Dan to speak to it.</t>
+          <t>• Other AI priorities the team is working on that I do not know about | Chris McComas, Chris Kostakis (2 min)
+• AI Discoverability | Alex Clemmons, Ethan Hanson (4 min)
+• AI Yields (content audit and enrichment for LLMO) | Markus Sheldon (4 min)
+• Design System Agentification (Create Hub, ties to the hub) | Dave Calleja (4 min)
+• Salesforce Agentic Harness | Markus Sheldon, Joe Anzalone (4 min)</t>
         </is>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>Dan Knauf</t>
+          <t>Chris McComas, Chris Kostakis, Alex Clemmons, Ethan Hanson, Markus Sheldon, Dave Calleja, Joe Anzalone</t>
         </is>
       </c>
       <c r="I13" s="13" t="inlineStr">
         <is>
-          <t>CTO</t>
+          <t>DBT</t>
         </is>
       </c>
       <c r="J13" s="13" t="inlineStr">
         <is>
-          <t>Click-down</t>
+          <t>Lightning updates</t>
         </is>
       </c>
       <c r="K13" s="13" t="inlineStr">
         <is>
-          <t>A short prompt slide.</t>
+          <t>What they already have: problem, how it is going, value, what it is built on, next steps and needs.</t>
         </is>
       </c>
       <c r="L13" s="13" t="inlineStr">
         <is>
-          <t>Shorten or send in writing</t>
+          <t>Shorten each to 3 min</t>
         </is>
       </c>
       <c r="M13" s="13" t="inlineStr">
         <is>
-          <t>You have not said what to cover on this one.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
+          <t>Markus Sheldon covers two items.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="101.25" customHeight="1">
       <c r="A14" s="10" t="n">
         <v>9</v>
       </c>
@@ -1134,41 +1143,43 @@
         <v/>
       </c>
       <c r="D14" s="10" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>2. Risk Review and priorities</t>
+          <t>6. AI DLC (DBT and DDM)</t>
         </is>
       </c>
       <c r="F14" s="12" t="inlineStr">
         <is>
-          <t>What the team is doing to speed up reviews</t>
+          <t>AI DLC: DBT and DDM together</t>
         </is>
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>People say this is going slowly. Update on the meeting Dan had with the Risk team, Shawn Street and Trisha.</t>
+          <t>• Callout: one of Pete's top priorities | Rachel Harris (1 min)
+• DBT: what has been done, the value it has added, where it is going, and what is shareable | Chris Kostakis (7 min)
+• DDM: where they see it going. Chris K. has a software delivery lifecycle framework for DBT; we are connecting with him to adopt the Claude-led process on other development teams, and gathering what is shareable | David Case, Robert Bush, Derelle Redmond (6 min)</t>
         </is>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>Dan Knauf, Trisha Scott</t>
+          <t>Rachel Harris, Chris Kostakis, David Case, Robert Bush, Derelle Redmond</t>
         </is>
       </c>
       <c r="I14" s="13" t="inlineStr">
         <is>
-          <t>CTO; Legal</t>
+          <t>Ops; DBT; DDM</t>
         </is>
       </c>
       <c r="J14" s="13" t="inlineStr">
         <is>
-          <t>Update</t>
+          <t>Presentations</t>
         </is>
       </c>
       <c r="K14" s="13" t="inlineStr">
         <is>
-          <t>A few bullets on the meetings.</t>
+          <t>A few slides (DBT). A few bullets or a slide (DDM).</t>
         </is>
       </c>
       <c r="L14" s="13" t="inlineStr">
@@ -1176,13 +1187,9 @@
           <t>Must keep</t>
         </is>
       </c>
-      <c r="M14" s="13" t="inlineStr">
-        <is>
-          <t>Shawn Street is not on the roster.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
+      <c r="M14" s="13" t="inlineStr"/>
+    </row>
+    <row r="15" ht="155.25" customHeight="1">
       <c r="A15" s="10" t="n">
         <v>10</v>
       </c>
@@ -1195,47 +1202,59 @@
         <v/>
       </c>
       <c r="D15" s="10" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>2. Risk Review and priorities</t>
+          <t>7. DDM</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>Ask 1: priorities we can raise in these calls</t>
+          <t>DDM</t>
         </is>
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>We need to start working on priorities we can surface in these calls, so we can prioritize requests and guide teams to focus on ours. Lots of things come in.</t>
+          <t>• Other AI priorities the team is working on that I do not know about | Deana Derocha, Stephen Meyer (2 min)
+• Client AI Operating Agreement, then discussion: pursue it? who wants to help? value for the group? | Stephen Meyer (5 min)
+• Measurement Framework and Reporting, then the same discussion | Stephen Meyer (5 min)
+• AI Decisioning: AI deciding individual customer journeys in CRM tools (for example Braze, Hightouch) | Barry Latimer (4 min)
+• ResTech and Synthetic Data: tools built, roadmap, synthetic data augments primary research and does not replace it; MCI exploring the same | Kartik Poduval, Christopher Cottam (4 min)</t>
         </is>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
-          <t>Dan Knauf, Trisha Scott</t>
+          <t>Deana Derocha, Stephen Meyer, Barry Latimer, Kartik Poduval, Christopher Cottam</t>
         </is>
       </c>
       <c r="I15" s="13" t="inlineStr">
         <is>
-          <t>CTO; Legal</t>
+          <t>DDM</t>
         </is>
       </c>
       <c r="J15" s="13" t="inlineStr">
         <is>
-          <t>Ask + discussion</t>
-        </is>
-      </c>
-      <c r="K15" s="13" t="inlineStr"/>
+          <t>Lightning updates + discussion</t>
+        </is>
+      </c>
+      <c r="K15" s="13" t="inlineStr">
+        <is>
+          <t>What they already have.</t>
+        </is>
+      </c>
       <c r="L15" s="13" t="inlineStr">
         <is>
-          <t>Must keep</t>
-        </is>
-      </c>
-      <c r="M15" s="13" t="inlineStr"/>
-    </row>
-    <row r="16">
+          <t>AI Decisioning and ResTech can go in writing</t>
+        </is>
+      </c>
+      <c r="M15" s="13" t="inlineStr">
+        <is>
+          <t>Barry to confirm the AI Decisioning description.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="47.25" customHeight="1">
       <c r="A16" s="10" t="n">
         <v>11</v>
       </c>
@@ -1248,52 +1267,52 @@
         <v/>
       </c>
       <c r="D16" s="10" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>2. Risk Review and priorities</t>
+          <t>8. Spotlight</t>
         </is>
       </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>Ask 2: how we show up when we enter requests</t>
+          <t>Spotlight: change management at the Google conference</t>
         </is>
       </c>
       <c r="G16" s="13" t="inlineStr">
         <is>
-          <t>• Example of a really good request, with the level of detail we need
-• If we want things to move quickly, the business side also has to respond quickly</t>
+          <t>• What Stephen heard about how Google handles change management (5 min)
+• Conversation: how it could apply to us (5 min)</t>
         </is>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>Dan Knauf, Trisha Scott</t>
+          <t>Stephen Meyer</t>
         </is>
       </c>
       <c r="I16" s="13" t="inlineStr">
         <is>
-          <t>CTO; Legal</t>
+          <t>DDM</t>
         </is>
       </c>
       <c r="J16" s="13" t="inlineStr">
         <is>
-          <t>Ask + discussion</t>
+          <t>Spotlight + discussion</t>
         </is>
       </c>
       <c r="K16" s="13" t="inlineStr">
         <is>
-          <t>One real example of a strong request (names removed if needed).</t>
+          <t>A few slides or notes.</t>
         </is>
       </c>
       <c r="L16" s="13" t="inlineStr">
         <is>
-          <t>Must keep</t>
+          <t>Shorten to 7 min</t>
         </is>
       </c>
       <c r="M16" s="13" t="inlineStr"/>
     </row>
-    <row r="17">
+    <row r="17" ht="114.75" customHeight="1">
       <c r="A17" s="10" t="n">
         <v>12</v>
       </c>
@@ -1306,52 +1325,59 @@
         <v/>
       </c>
       <c r="D17" s="10" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>3. AI market moves</t>
+          <t>9. Business groups</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>Quick pulse on what competitors are doing with AI</t>
+          <t>Business groups</t>
         </is>
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>• Quick pulse on what competitors are doing specifically with AI
-• Discussion: ideas we could use, things we could learn</t>
+          <t>• Client &amp; Commercial: tools, initiatives and similar | Mike Monacelli (5 min)
+• AI Commercial guidance: a teaser of where it is going | Alex Willard (3 min)
+• Solutioning: open slot, anything to share? | Tony Toubia (2 min)
+• AI Advisory: open slot, anything to share? | Jason Van Peeren (2 min)
+• Romulus: quick walkthrough | Adam Organ (5 min)</t>
         </is>
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
-          <t>Katherine Jones-Siemsen</t>
+          <t>Mike Monacelli, Alex Willard, Tony Toubia, Jason Van Peeren, Adam Organ</t>
         </is>
       </c>
       <c r="I17" s="13" t="inlineStr">
         <is>
-          <t>Strategy</t>
+          <t>Client &amp; Commercial; Finance; Solutioning; AI Advisory; Not on roster</t>
         </is>
       </c>
       <c r="J17" s="13" t="inlineStr">
         <is>
-          <t>Update + discussion</t>
+          <t>Updates + demo</t>
         </is>
       </c>
       <c r="K17" s="13" t="inlineStr">
         <is>
-          <t>A few slides or a one-page summary.</t>
+          <t>Mike: what they have. Alex: light teaser. Tony and Jason: only if there is something. Adam: a quick demo or recording.</t>
         </is>
       </c>
       <c r="L17" s="13" t="inlineStr">
         <is>
-          <t>Shorten to 5 min</t>
-        </is>
-      </c>
-      <c r="M17" s="13" t="inlineStr"/>
-    </row>
-    <row r="18">
+          <t>Skip Solutioning and AI Advisory if nothing to share; Mike and Adam to 3 min</t>
+        </is>
+      </c>
+      <c r="M17" s="13" t="inlineStr">
+        <is>
+          <t>Adam Organ is not on the roster.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="87.75" customHeight="1">
       <c r="A18" s="10" t="n">
         <v>13</v>
       </c>
@@ -1364,1382 +1390,61 @@
         <v/>
       </c>
       <c r="D18" s="10" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>4. Best practice hub</t>
+          <t>10. Close</t>
         </is>
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Vision for the hub (open discussion)</t>
+          <t>Knowledge management, open forum, news</t>
         </is>
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t>• We do not have the hub yet. Create Hub has started it, and it is our framework to get kicked off (see Design System Agentification)
-• Vision: one place for skills, plugins, connectors and shared context, tagged by role and craft
-• Open discussion: where we see it going, and the value across the org</t>
+          <t>• Knowledge management teaser: standing up a workforce. Raise hands to see who wants to help (3 min)
+• Open forum: need help? built something cool? Plus the open call: a big problem, something cool, or a team worth showcasing (4 min)
+• In the news (hot AI things) and announcements (Merkle/dentsu, trainings) (4 min)</t>
         </is>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>Dan Knauf, Dave Brabec</t>
+          <t>Rachel Harris</t>
         </is>
       </c>
       <c r="I18" s="13" t="inlineStr">
         <is>
-          <t>CTO; Ops</t>
+          <t>Ops</t>
         </is>
       </c>
       <c r="J18" s="13" t="inlineStr">
         <is>
-          <t>Presentation + discussion</t>
+          <t>Teaser, forum, updates</t>
         </is>
       </c>
       <c r="K18" s="13" t="inlineStr">
         <is>
-          <t>A few slides.</t>
+          <t>Open call collected in the pre-meet beforehand.</t>
         </is>
       </c>
       <c r="L18" s="13" t="inlineStr">
         <is>
-          <t>Must keep</t>
-        </is>
-      </c>
-      <c r="M18" s="13" t="inlineStr">
-        <is>
-          <t>Line up with Dave Calleja, who covers Design System Agentification later.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B19" s="7">
-        <f>C18</f>
-        <v/>
-      </c>
-      <c r="C19" s="7">
-        <f>B19+D19/1440</f>
-        <v/>
-      </c>
-      <c r="D19" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>Break</t>
-        </is>
-      </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>Break</t>
-        </is>
-      </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>Stretch and refill. If we are running late, shorten to 5 minutes.</t>
-        </is>
-      </c>
-      <c r="H19" s="9" t="inlineStr">
-        <is>
-          <t>Rachel Harris</t>
-        </is>
-      </c>
-      <c r="I19" s="9" t="inlineStr">
-        <is>
-          <t>Ops</t>
-        </is>
-      </c>
-      <c r="J19" s="9" t="inlineStr">
-        <is>
-          <t>Break</t>
-        </is>
-      </c>
-      <c r="K19" s="9" t="inlineStr"/>
-      <c r="L19" s="9" t="inlineStr">
-        <is>
-          <t>Shorten to 5 min</t>
-        </is>
-      </c>
-      <c r="M19" s="9" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="n">
-        <v>15</v>
-      </c>
-      <c r="B20" s="11">
-        <f>C19</f>
-        <v/>
-      </c>
-      <c r="C20" s="11">
-        <f>B20+D20/1440</f>
-        <v/>
-      </c>
-      <c r="D20" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E20" s="12" t="inlineStr">
-        <is>
-          <t>5. DBT</t>
-        </is>
-      </c>
-      <c r="F20" s="12" t="inlineStr">
-        <is>
-          <t>DBT: other AI priorities</t>
-        </is>
-      </c>
-      <c r="G20" s="13" t="inlineStr">
-        <is>
-          <t>Open ask: other AI priorities the team is working on that I do not know about and that could matter to the group.</t>
-        </is>
-      </c>
-      <c r="H20" s="13" t="inlineStr">
-        <is>
-          <t>Chris McComas, Chris Kostakis</t>
-        </is>
-      </c>
-      <c r="I20" s="13" t="inlineStr">
-        <is>
-          <t>DBT</t>
-        </is>
-      </c>
-      <c r="J20" s="13" t="inlineStr">
-        <is>
-          <t>Open ask</t>
-        </is>
-      </c>
-      <c r="K20" s="13" t="inlineStr">
-        <is>
-          <t>Passed to the team by the DBT leads.</t>
-        </is>
-      </c>
-      <c r="L20" s="13" t="inlineStr">
-        <is>
-          <t>Shorten</t>
-        </is>
-      </c>
-      <c r="M20" s="13" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="B21" s="11">
-        <f>C20</f>
-        <v/>
-      </c>
-      <c r="C21" s="11">
-        <f>B21+D21/1440</f>
-        <v/>
-      </c>
-      <c r="D21" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E21" s="12" t="inlineStr">
-        <is>
-          <t>5. DBT</t>
-        </is>
-      </c>
-      <c r="F21" s="12" t="inlineStr">
-        <is>
-          <t>AI Discoverability</t>
-        </is>
-      </c>
-      <c r="G21" s="13" t="inlineStr">
-        <is>
-          <t>Lightning update: problem, how it is going, value, what it is built on, next steps and what is needed.</t>
-        </is>
-      </c>
-      <c r="H21" s="13" t="inlineStr">
-        <is>
-          <t>Alex Clemmons, Ethan Hanson</t>
-        </is>
-      </c>
-      <c r="I21" s="13" t="inlineStr">
-        <is>
-          <t>DBT</t>
-        </is>
-      </c>
-      <c r="J21" s="13" t="inlineStr">
-        <is>
-          <t>Lightning update</t>
-        </is>
-      </c>
-      <c r="K21" s="13" t="inlineStr">
-        <is>
-          <t>What they already have.</t>
-        </is>
-      </c>
-      <c r="L21" s="13" t="inlineStr">
-        <is>
-          <t>Shorten to 3 min</t>
-        </is>
-      </c>
-      <c r="M21" s="13" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="10" t="n">
-        <v>17</v>
-      </c>
-      <c r="B22" s="11">
-        <f>C21</f>
-        <v/>
-      </c>
-      <c r="C22" s="11">
-        <f>B22+D22/1440</f>
-        <v/>
-      </c>
-      <c r="D22" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E22" s="12" t="inlineStr">
-        <is>
-          <t>5. DBT</t>
-        </is>
-      </c>
-      <c r="F22" s="12" t="inlineStr">
-        <is>
-          <t>AI Yields (content audit and enrichment for LLMO)</t>
-        </is>
-      </c>
-      <c r="G22" s="13" t="inlineStr">
-        <is>
-          <t>Lightning update: problem, how it is going, value, what it is built on, next steps and what is needed.</t>
-        </is>
-      </c>
-      <c r="H22" s="13" t="inlineStr">
-        <is>
-          <t>Markus Sheldon</t>
-        </is>
-      </c>
-      <c r="I22" s="13" t="inlineStr">
-        <is>
-          <t>DBT</t>
-        </is>
-      </c>
-      <c r="J22" s="13" t="inlineStr">
-        <is>
-          <t>Lightning update</t>
-        </is>
-      </c>
-      <c r="K22" s="13" t="inlineStr">
-        <is>
-          <t>What they already have.</t>
-        </is>
-      </c>
-      <c r="L22" s="13" t="inlineStr">
-        <is>
-          <t>Shorten to 3 min</t>
-        </is>
-      </c>
-      <c r="M22" s="13" t="inlineStr">
-        <is>
-          <t>Markus also covers the Salesforce Agentic Harness.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="10" t="n">
-        <v>18</v>
-      </c>
-      <c r="B23" s="11">
-        <f>C22</f>
-        <v/>
-      </c>
-      <c r="C23" s="11">
-        <f>B23+D23/1440</f>
-        <v/>
-      </c>
-      <c r="D23" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E23" s="12" t="inlineStr">
-        <is>
-          <t>5. DBT</t>
-        </is>
-      </c>
-      <c r="F23" s="12" t="inlineStr">
-        <is>
-          <t>Design System Agentification</t>
-        </is>
-      </c>
-      <c r="G23" s="13" t="inlineStr">
-        <is>
-          <t>Lightning update. Create Hub has started the hub, so connect this to the Best practice hub segment.</t>
-        </is>
-      </c>
-      <c r="H23" s="13" t="inlineStr">
-        <is>
-          <t>Dave Calleja</t>
-        </is>
-      </c>
-      <c r="I23" s="13" t="inlineStr">
-        <is>
-          <t>DBT</t>
-        </is>
-      </c>
-      <c r="J23" s="13" t="inlineStr">
-        <is>
-          <t>Lightning update</t>
-        </is>
-      </c>
-      <c r="K23" s="13" t="inlineStr">
-        <is>
-          <t>What they already have.</t>
-        </is>
-      </c>
-      <c r="L23" s="13" t="inlineStr">
-        <is>
-          <t>Must keep</t>
-        </is>
-      </c>
-      <c r="M23" s="13" t="inlineStr">
-        <is>
-          <t>Ties to the Best practice hub.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="n">
-        <v>19</v>
-      </c>
-      <c r="B24" s="11">
-        <f>C23</f>
-        <v/>
-      </c>
-      <c r="C24" s="11">
-        <f>B24+D24/1440</f>
-        <v/>
-      </c>
-      <c r="D24" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E24" s="12" t="inlineStr">
-        <is>
-          <t>5. DBT</t>
-        </is>
-      </c>
-      <c r="F24" s="12" t="inlineStr">
-        <is>
-          <t>Salesforce Agentic Harness</t>
-        </is>
-      </c>
-      <c r="G24" s="13" t="inlineStr">
-        <is>
-          <t>Lightning update: problem, how it is going, value, what it is built on, next steps and what is needed.</t>
-        </is>
-      </c>
-      <c r="H24" s="13" t="inlineStr">
-        <is>
-          <t>Markus Sheldon, Joe Anzalone</t>
-        </is>
-      </c>
-      <c r="I24" s="13" t="inlineStr">
-        <is>
-          <t>DBT</t>
-        </is>
-      </c>
-      <c r="J24" s="13" t="inlineStr">
-        <is>
-          <t>Lightning update</t>
-        </is>
-      </c>
-      <c r="K24" s="13" t="inlineStr">
-        <is>
-          <t>What they already have.</t>
-        </is>
-      </c>
-      <c r="L24" s="13" t="inlineStr">
-        <is>
-          <t>Shorten to 3 min</t>
-        </is>
-      </c>
-      <c r="M24" s="13" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="B25" s="11">
-        <f>C24</f>
-        <v/>
-      </c>
-      <c r="C25" s="11">
-        <f>B25+D25/1440</f>
-        <v/>
-      </c>
-      <c r="D25" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="12" t="inlineStr">
-        <is>
-          <t>6. AI DLC (DBT and DDM)</t>
-        </is>
-      </c>
-      <c r="F25" s="12" t="inlineStr">
-        <is>
-          <t>Callout: one of Pete's top priorities</t>
-        </is>
-      </c>
-      <c r="G25" s="13" t="inlineStr">
-        <is>
-          <t>Why this one matters, then hand to DBT and DDM.</t>
-        </is>
-      </c>
-      <c r="H25" s="13" t="inlineStr">
-        <is>
-          <t>Rachel Harris</t>
-        </is>
-      </c>
-      <c r="I25" s="13" t="inlineStr">
-        <is>
-          <t>Ops</t>
-        </is>
-      </c>
-      <c r="J25" s="13" t="inlineStr">
-        <is>
-          <t>Callout</t>
-        </is>
-      </c>
-      <c r="K25" s="13" t="inlineStr"/>
-      <c r="L25" s="13" t="inlineStr">
-        <is>
-          <t>Must keep</t>
-        </is>
-      </c>
-      <c r="M25" s="13" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="n">
-        <v>21</v>
-      </c>
-      <c r="B26" s="11">
-        <f>C25</f>
-        <v/>
-      </c>
-      <c r="C26" s="11">
-        <f>B26+D26/1440</f>
-        <v/>
-      </c>
-      <c r="D26" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="E26" s="12" t="inlineStr">
-        <is>
-          <t>6. AI DLC (DBT and DDM)</t>
-        </is>
-      </c>
-      <c r="F26" s="12" t="inlineStr">
-        <is>
-          <t>DBT: what has been done and where it is going</t>
-        </is>
-      </c>
-      <c r="G26" s="13" t="inlineStr">
-        <is>
-          <t>• What has already been done
-• The value it has been adding
-• Where we see it going
-• What is shareable</t>
-        </is>
-      </c>
-      <c r="H26" s="13" t="inlineStr">
-        <is>
-          <t>Chris Kostakis</t>
-        </is>
-      </c>
-      <c r="I26" s="13" t="inlineStr">
-        <is>
-          <t>DBT</t>
-        </is>
-      </c>
-      <c r="J26" s="13" t="inlineStr">
-        <is>
-          <t>Presentation</t>
-        </is>
-      </c>
-      <c r="K26" s="13" t="inlineStr">
-        <is>
-          <t>A few slides.</t>
-        </is>
-      </c>
-      <c r="L26" s="13" t="inlineStr">
-        <is>
-          <t>Must keep</t>
-        </is>
-      </c>
-      <c r="M26" s="13" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="10" t="n">
-        <v>22</v>
-      </c>
-      <c r="B27" s="11">
-        <f>C26</f>
-        <v/>
-      </c>
-      <c r="C27" s="11">
-        <f>B27+D27/1440</f>
-        <v/>
-      </c>
-      <c r="D27" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E27" s="12" t="inlineStr">
-        <is>
-          <t>6. AI DLC (DBT and DDM)</t>
-        </is>
-      </c>
-      <c r="F27" s="12" t="inlineStr">
-        <is>
-          <t>DDM: where they see it going</t>
-        </is>
-      </c>
-      <c r="G27" s="13" t="inlineStr">
-        <is>
-          <t>• Chris K. has a software delivery lifecycle framework for DBT
-• We are connecting with him to see if we can adopt that Claude-led process on our other development teams
-• Right now we are gathering what is shareable</t>
-        </is>
-      </c>
-      <c r="H27" s="13" t="inlineStr">
-        <is>
-          <t>David Case, Robert Bush, Derelle Redmond</t>
-        </is>
-      </c>
-      <c r="I27" s="13" t="inlineStr">
-        <is>
-          <t>DDM</t>
-        </is>
-      </c>
-      <c r="J27" s="13" t="inlineStr">
-        <is>
-          <t>Presentation</t>
-        </is>
-      </c>
-      <c r="K27" s="13" t="inlineStr">
-        <is>
-          <t>A few bullets or a slide.</t>
-        </is>
-      </c>
-      <c r="L27" s="13" t="inlineStr">
-        <is>
-          <t>Must keep</t>
-        </is>
-      </c>
-      <c r="M27" s="13" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="10" t="n">
-        <v>23</v>
-      </c>
-      <c r="B28" s="11">
-        <f>C27</f>
-        <v/>
-      </c>
-      <c r="C28" s="11">
-        <f>B28+D28/1440</f>
-        <v/>
-      </c>
-      <c r="D28" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E28" s="12" t="inlineStr">
-        <is>
-          <t>7. DDM</t>
-        </is>
-      </c>
-      <c r="F28" s="12" t="inlineStr">
-        <is>
-          <t>DDM: other AI priorities</t>
-        </is>
-      </c>
-      <c r="G28" s="13" t="inlineStr">
-        <is>
-          <t>Open ask: other AI priorities the team is working on that I do not know about.</t>
-        </is>
-      </c>
-      <c r="H28" s="13" t="inlineStr">
-        <is>
-          <t>Deana Derocha, Stephen Meyer</t>
-        </is>
-      </c>
-      <c r="I28" s="13" t="inlineStr">
-        <is>
-          <t>DDM</t>
-        </is>
-      </c>
-      <c r="J28" s="13" t="inlineStr">
-        <is>
-          <t>Open ask</t>
-        </is>
-      </c>
-      <c r="K28" s="13" t="inlineStr">
-        <is>
-          <t>Passed to the team by the DDM leads.</t>
-        </is>
-      </c>
-      <c r="L28" s="13" t="inlineStr">
-        <is>
-          <t>Shorten</t>
-        </is>
-      </c>
-      <c r="M28" s="13" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="10" t="n">
-        <v>24</v>
-      </c>
-      <c r="B29" s="11">
-        <f>C28</f>
-        <v/>
-      </c>
-      <c r="C29" s="11">
-        <f>B29+D29/1440</f>
-        <v/>
-      </c>
-      <c r="D29" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E29" s="12" t="inlineStr">
-        <is>
-          <t>7. DDM</t>
-        </is>
-      </c>
-      <c r="F29" s="12" t="inlineStr">
-        <is>
-          <t>Client AI Operating Agreement</t>
-        </is>
-      </c>
-      <c r="G29" s="13" t="inlineStr">
-        <is>
-          <t>Then an open discussion: should we pursue this, who wants to help, and what is the value for the whole group?</t>
-        </is>
-      </c>
-      <c r="H29" s="13" t="inlineStr">
-        <is>
-          <t>Stephen Meyer</t>
-        </is>
-      </c>
-      <c r="I29" s="13" t="inlineStr">
-        <is>
-          <t>DDM</t>
-        </is>
-      </c>
-      <c r="J29" s="13" t="inlineStr">
-        <is>
-          <t>Update + discussion</t>
-        </is>
-      </c>
-      <c r="K29" s="13" t="inlineStr">
-        <is>
-          <t>What they already have.</t>
-        </is>
-      </c>
-      <c r="L29" s="13" t="inlineStr">
-        <is>
-          <t>Shorten to 4 min</t>
-        </is>
-      </c>
-      <c r="M29" s="13" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="10" t="n">
-        <v>25</v>
-      </c>
-      <c r="B30" s="11">
-        <f>C29</f>
-        <v/>
-      </c>
-      <c r="C30" s="11">
-        <f>B30+D30/1440</f>
-        <v/>
-      </c>
-      <c r="D30" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E30" s="12" t="inlineStr">
-        <is>
-          <t>7. DDM</t>
-        </is>
-      </c>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>Measurement Framework and Reporting</t>
-        </is>
-      </c>
-      <c r="G30" s="13" t="inlineStr">
-        <is>
-          <t>Then an open discussion: should we pursue this, who wants to help, and what is the value for the whole group?</t>
-        </is>
-      </c>
-      <c r="H30" s="13" t="inlineStr">
-        <is>
-          <t>Stephen Meyer</t>
-        </is>
-      </c>
-      <c r="I30" s="13" t="inlineStr">
-        <is>
-          <t>DDM</t>
-        </is>
-      </c>
-      <c r="J30" s="13" t="inlineStr">
-        <is>
-          <t>Update + discussion</t>
-        </is>
-      </c>
-      <c r="K30" s="13" t="inlineStr">
-        <is>
-          <t>What they already have.</t>
-        </is>
-      </c>
-      <c r="L30" s="13" t="inlineStr">
-        <is>
-          <t>Shorten to 4 min</t>
-        </is>
-      </c>
-      <c r="M30" s="13" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="10" t="n">
-        <v>26</v>
-      </c>
-      <c r="B31" s="11">
-        <f>C30</f>
-        <v/>
-      </c>
-      <c r="C31" s="11">
-        <f>B31+D31/1440</f>
-        <v/>
-      </c>
-      <c r="D31" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E31" s="12" t="inlineStr">
-        <is>
-          <t>7. DDM</t>
-        </is>
-      </c>
-      <c r="F31" s="12" t="inlineStr">
-        <is>
-          <t>AI Decisioning</t>
-        </is>
-      </c>
-      <c r="G31" s="13" t="inlineStr">
-        <is>
-          <t>AI deciding individual customer journeys inside CRM tools (for example Braze and Hightouch): one email, two SMS and one in-app message for one person, instead of fully planned campaigns.</t>
-        </is>
-      </c>
-      <c r="H31" s="13" t="inlineStr">
-        <is>
-          <t>Barry Latimer</t>
-        </is>
-      </c>
-      <c r="I31" s="13" t="inlineStr">
-        <is>
-          <t>DDM</t>
-        </is>
-      </c>
-      <c r="J31" s="13" t="inlineStr">
-        <is>
-          <t>Lightning update</t>
-        </is>
-      </c>
-      <c r="K31" s="13" t="inlineStr">
-        <is>
-          <t>A short explanation.</t>
-        </is>
-      </c>
-      <c r="L31" s="13" t="inlineStr">
-        <is>
-          <t>Can cut or send in writing</t>
-        </is>
-      </c>
-      <c r="M31" s="13" t="inlineStr">
-        <is>
-          <t>Barry to confirm the description.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="B32" s="11">
-        <f>C31</f>
-        <v/>
-      </c>
-      <c r="C32" s="11">
-        <f>B32+D32/1440</f>
-        <v/>
-      </c>
-      <c r="D32" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E32" s="12" t="inlineStr">
-        <is>
-          <t>7. DDM</t>
-        </is>
-      </c>
-      <c r="F32" s="12" t="inlineStr">
-        <is>
-          <t>ResTech and Synthetic Data</t>
-        </is>
-      </c>
-      <c r="G32" s="13" t="inlineStr">
-        <is>
-          <t>• Tools the market research team has built, and what is on the roadmap
-• Synthetic data augments primary research and does not replace it; researchers still validate how close synthetic respondents are to real ones
-• MCI is exploring the same idea (synthetic personas, synthetic datasets for prototyping)</t>
-        </is>
-      </c>
-      <c r="H32" s="13" t="inlineStr">
-        <is>
-          <t>Kartik Poduval, Christopher Cottam</t>
-        </is>
-      </c>
-      <c r="I32" s="13" t="inlineStr">
-        <is>
-          <t>DDM</t>
-        </is>
-      </c>
-      <c r="J32" s="13" t="inlineStr">
-        <is>
-          <t>Lightning update</t>
-        </is>
-      </c>
-      <c r="K32" s="13" t="inlineStr">
-        <is>
-          <t>What they already have.</t>
-        </is>
-      </c>
-      <c r="L32" s="13" t="inlineStr">
-        <is>
-          <t>Can cut or send in writing</t>
-        </is>
-      </c>
-      <c r="M32" s="13" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="10" t="n">
-        <v>28</v>
-      </c>
-      <c r="B33" s="11">
-        <f>C32</f>
-        <v/>
-      </c>
-      <c r="C33" s="11">
-        <f>B33+D33/1440</f>
-        <v/>
-      </c>
-      <c r="D33" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="E33" s="12" t="inlineStr">
-        <is>
-          <t>8. Spotlight</t>
-        </is>
-      </c>
-      <c r="F33" s="12" t="inlineStr">
-        <is>
-          <t>Change management: what Google shared</t>
-        </is>
-      </c>
-      <c r="G33" s="13" t="inlineStr">
-        <is>
-          <t>• What Stephen heard at the Google conference about how Google handles change management
-• Conversation: how it could apply to us</t>
-        </is>
-      </c>
-      <c r="H33" s="13" t="inlineStr">
-        <is>
-          <t>Stephen Meyer</t>
-        </is>
-      </c>
-      <c r="I33" s="13" t="inlineStr">
-        <is>
-          <t>DDM</t>
-        </is>
-      </c>
-      <c r="J33" s="13" t="inlineStr">
-        <is>
-          <t>Spotlight + discussion</t>
-        </is>
-      </c>
-      <c r="K33" s="13" t="inlineStr">
-        <is>
-          <t>A few slides or notes.</t>
-        </is>
-      </c>
-      <c r="L33" s="13" t="inlineStr">
-        <is>
-          <t>Shorten to 7 min</t>
-        </is>
-      </c>
-      <c r="M33" s="13" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="10" t="n">
-        <v>29</v>
-      </c>
-      <c r="B34" s="11">
-        <f>C33</f>
-        <v/>
-      </c>
-      <c r="C34" s="11">
-        <f>B34+D34/1440</f>
-        <v/>
-      </c>
-      <c r="D34" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="E34" s="12" t="inlineStr">
-        <is>
-          <t>9. Business groups</t>
-        </is>
-      </c>
-      <c r="F34" s="12" t="inlineStr">
-        <is>
-          <t>Client &amp; Commercial</t>
-        </is>
-      </c>
-      <c r="G34" s="13" t="inlineStr">
-        <is>
-          <t>Tools, initiatives and similar.</t>
-        </is>
-      </c>
-      <c r="H34" s="13" t="inlineStr">
-        <is>
-          <t>Mike Monacelli</t>
-        </is>
-      </c>
-      <c r="I34" s="13" t="inlineStr">
-        <is>
-          <t>Client &amp; Commercial</t>
-        </is>
-      </c>
-      <c r="J34" s="13" t="inlineStr">
-        <is>
-          <t>Update</t>
-        </is>
-      </c>
-      <c r="K34" s="13" t="inlineStr">
-        <is>
-          <t>What they already have.</t>
-        </is>
-      </c>
-      <c r="L34" s="13" t="inlineStr">
-        <is>
-          <t>Shorten to 3 min</t>
-        </is>
-      </c>
-      <c r="M34" s="13" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="10" t="n">
-        <v>30</v>
-      </c>
-      <c r="B35" s="11">
-        <f>C34</f>
-        <v/>
-      </c>
-      <c r="C35" s="11">
-        <f>B35+D35/1440</f>
-        <v/>
-      </c>
-      <c r="D35" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E35" s="12" t="inlineStr">
-        <is>
-          <t>9. Business groups</t>
-        </is>
-      </c>
-      <c r="F35" s="12" t="inlineStr">
-        <is>
-          <t>AI Commercial guidance (teaser)</t>
-        </is>
-      </c>
-      <c r="G35" s="13" t="inlineStr">
-        <is>
-          <t>A teaser of where this is going.</t>
-        </is>
-      </c>
-      <c r="H35" s="13" t="inlineStr">
-        <is>
-          <t>Alex Willard</t>
-        </is>
-      </c>
-      <c r="I35" s="13" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="J35" s="13" t="inlineStr">
-        <is>
-          <t>Teaser</t>
-        </is>
-      </c>
-      <c r="K35" s="13" t="inlineStr">
-        <is>
-          <t>Light. Where it is headed.</t>
-        </is>
-      </c>
-      <c r="L35" s="13" t="inlineStr">
-        <is>
-          <t>Shorten</t>
-        </is>
-      </c>
-      <c r="M35" s="13" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="10" t="n">
-        <v>31</v>
-      </c>
-      <c r="B36" s="11">
-        <f>C35</f>
-        <v/>
-      </c>
-      <c r="C36" s="11">
-        <f>B36+D36/1440</f>
-        <v/>
-      </c>
-      <c r="D36" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E36" s="12" t="inlineStr">
-        <is>
-          <t>9. Business groups</t>
-        </is>
-      </c>
-      <c r="F36" s="12" t="inlineStr">
-        <is>
-          <t>Solutioning</t>
-        </is>
-      </c>
-      <c r="G36" s="13" t="inlineStr">
-        <is>
-          <t>Open slot: anything to share?</t>
-        </is>
-      </c>
-      <c r="H36" s="13" t="inlineStr">
-        <is>
-          <t>Tony Toubia</t>
-        </is>
-      </c>
-      <c r="I36" s="13" t="inlineStr">
-        <is>
-          <t>Solutioning</t>
-        </is>
-      </c>
-      <c r="J36" s="13" t="inlineStr">
-        <is>
-          <t>Open slot</t>
-        </is>
-      </c>
-      <c r="K36" s="13" t="inlineStr">
-        <is>
-          <t>Only if there is something.</t>
-        </is>
-      </c>
-      <c r="L36" s="13" t="inlineStr">
-        <is>
-          <t>Can cut if nothing to share</t>
-        </is>
-      </c>
-      <c r="M36" s="13" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="10" t="n">
-        <v>32</v>
-      </c>
-      <c r="B37" s="11">
-        <f>C36</f>
-        <v/>
-      </c>
-      <c r="C37" s="11">
-        <f>B37+D37/1440</f>
-        <v/>
-      </c>
-      <c r="D37" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E37" s="12" t="inlineStr">
-        <is>
-          <t>9. Business groups</t>
-        </is>
-      </c>
-      <c r="F37" s="12" t="inlineStr">
-        <is>
-          <t>AI Advisory</t>
-        </is>
-      </c>
-      <c r="G37" s="13" t="inlineStr">
-        <is>
-          <t>Open slot: anything to share?</t>
-        </is>
-      </c>
-      <c r="H37" s="13" t="inlineStr">
-        <is>
-          <t>Jason Van Peeren</t>
-        </is>
-      </c>
-      <c r="I37" s="13" t="inlineStr">
-        <is>
-          <t>AI Advisory</t>
-        </is>
-      </c>
-      <c r="J37" s="13" t="inlineStr">
-        <is>
-          <t>Open slot</t>
-        </is>
-      </c>
-      <c r="K37" s="13" t="inlineStr">
-        <is>
-          <t>Only if there is something.</t>
-        </is>
-      </c>
-      <c r="L37" s="13" t="inlineStr">
-        <is>
-          <t>Can cut if nothing to share</t>
-        </is>
-      </c>
-      <c r="M37" s="13" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="10" t="n">
-        <v>33</v>
-      </c>
-      <c r="B38" s="11">
-        <f>C37</f>
-        <v/>
-      </c>
-      <c r="C38" s="11">
-        <f>B38+D38/1440</f>
-        <v/>
-      </c>
-      <c r="D38" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="E38" s="12" t="inlineStr">
-        <is>
-          <t>9. Business groups</t>
-        </is>
-      </c>
-      <c r="F38" s="12" t="inlineStr">
-        <is>
-          <t>Romulus walkthrough</t>
-        </is>
-      </c>
-      <c r="G38" s="13" t="inlineStr">
-        <is>
-          <t>Quick walkthrough, live or recorded.</t>
-        </is>
-      </c>
-      <c r="H38" s="13" t="inlineStr">
-        <is>
-          <t>Adam Organ</t>
-        </is>
-      </c>
-      <c r="I38" s="13" t="inlineStr">
-        <is>
-          <t>Not on roster</t>
-        </is>
-      </c>
-      <c r="J38" s="13" t="inlineStr">
-        <is>
-          <t>Demo</t>
-        </is>
-      </c>
-      <c r="K38" s="13" t="inlineStr">
-        <is>
-          <t>A quick demo or screen recording.</t>
-        </is>
-      </c>
-      <c r="L38" s="13" t="inlineStr">
-        <is>
-          <t>Shorten to 3 min</t>
-        </is>
-      </c>
-      <c r="M38" s="13" t="inlineStr">
-        <is>
-          <t>Adam Organ is not on the roster.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="B39" s="11">
-        <f>C38</f>
-        <v/>
-      </c>
-      <c r="C39" s="11">
-        <f>B39+D39/1440</f>
-        <v/>
-      </c>
-      <c r="D39" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E39" s="12" t="inlineStr">
-        <is>
-          <t>10. Knowledge management</t>
-        </is>
-      </c>
-      <c r="F39" s="12" t="inlineStr">
-        <is>
-          <t>Teaser: standing up a workforce</t>
-        </is>
-      </c>
-      <c r="G39" s="13" t="inlineStr">
-        <is>
-          <t>A teaser, then raise hands to see who wants to help figure this out.</t>
-        </is>
-      </c>
-      <c r="H39" s="13" t="inlineStr">
-        <is>
-          <t>Rachel Harris</t>
-        </is>
-      </c>
-      <c r="I39" s="13" t="inlineStr">
-        <is>
-          <t>Ops</t>
-        </is>
-      </c>
-      <c r="J39" s="13" t="inlineStr">
-        <is>
-          <t>Teaser + ask</t>
-        </is>
-      </c>
-      <c r="K39" s="13" t="inlineStr"/>
-      <c r="L39" s="13" t="inlineStr">
-        <is>
-          <t>Shorten</t>
-        </is>
-      </c>
-      <c r="M39" s="13" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="10" t="n">
-        <v>35</v>
-      </c>
-      <c r="B40" s="11">
-        <f>C39</f>
-        <v/>
-      </c>
-      <c r="C40" s="11">
-        <f>B40+D40/1440</f>
-        <v/>
-      </c>
-      <c r="D40" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E40" s="12" t="inlineStr">
-        <is>
-          <t>11. Close</t>
-        </is>
-      </c>
-      <c r="F40" s="12" t="inlineStr">
-        <is>
-          <t>Open forum</t>
-        </is>
-      </c>
-      <c r="G40" s="13" t="inlineStr">
-        <is>
-          <t>• Need help with something? Ask the room
-• Has anyone built something really cool they want to share?
-• Open call: a big problem, something cool, or a team worth showcasing</t>
-        </is>
-      </c>
-      <c r="H40" s="13" t="inlineStr">
-        <is>
-          <t>Rachel Harris</t>
-        </is>
-      </c>
-      <c r="I40" s="13" t="inlineStr">
-        <is>
-          <t>Ops</t>
-        </is>
-      </c>
-      <c r="J40" s="13" t="inlineStr">
-        <is>
-          <t>Open forum</t>
-        </is>
-      </c>
-      <c r="K40" s="13" t="inlineStr">
-        <is>
-          <t>Collected in the pre-meet beforehand.</t>
-        </is>
-      </c>
-      <c r="L40" s="13" t="inlineStr">
-        <is>
-          <t>Can move to the weekly meeting</t>
-        </is>
-      </c>
-      <c r="M40" s="13" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="10" t="n">
-        <v>36</v>
-      </c>
-      <c r="B41" s="11">
-        <f>C40</f>
-        <v/>
-      </c>
-      <c r="C41" s="11">
-        <f>B41+D41/1440</f>
-        <v/>
-      </c>
-      <c r="D41" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E41" s="12" t="inlineStr">
-        <is>
-          <t>11. Close</t>
-        </is>
-      </c>
-      <c r="F41" s="12" t="inlineStr">
-        <is>
-          <t>In the news and announcements</t>
-        </is>
-      </c>
-      <c r="G41" s="13" t="inlineStr">
-        <is>
-          <t>• In the news: hot AI things
-• Other announcements: Merkle/dentsu, trainings</t>
-        </is>
-      </c>
-      <c r="H41" s="13" t="inlineStr">
-        <is>
-          <t>Rachel Harris</t>
-        </is>
-      </c>
-      <c r="I41" s="13" t="inlineStr">
-        <is>
-          <t>Ops</t>
-        </is>
-      </c>
-      <c r="J41" s="13" t="inlineStr">
-        <is>
-          <t>Update</t>
-        </is>
-      </c>
-      <c r="K41" s="13" t="inlineStr"/>
-      <c r="L41" s="13" t="inlineStr">
-        <is>
-          <t>Can send in writing</t>
-        </is>
-      </c>
-      <c r="M41" s="13" t="inlineStr"/>
+          <t>Open forum to the weekly meeting; news in writing</t>
+        </is>
+      </c>
+      <c r="M18" s="13" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A5:M41"/>
+  <autoFilter ref="A5:M18"/>
+  <mergeCells count="2">
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A2:B2"/>
+  </mergeCells>
   <dataValidations count="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2872,7 +1577,7 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>Shorten the fireside chat from 10 to 6 minutes</t>
+          <t>Shorten the fireside chat from 12 to 8 minutes</t>
         </is>
       </c>
       <c r="C8" s="13" t="n">

</xml_diff>

<commit_message>
Agenda: user's timings plus 10 min to groups and open items
</commit_message>
<xml_diff>
--- a/AI_Steerco_Kickoff_Agenda.xlsx
+++ b/AI_Steerco_Kickoff_Agenda.xlsx
@@ -841,7 +841,7 @@
         <v/>
       </c>
       <c r="D9" s="10" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
@@ -855,9 +855,9 @@
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>• What the team is doing to speed up reviews: update on the meeting Dan had with the Risk team, Shawn Street and Trisha (4 min)
-• Ask 1: start working on priorities we can surface in these calls, so we can prioritize requests and guide teams to ours (lots of things come in) (5 min)
-• Ask 2: how we show up when entering requests. Example of a really good request; if we want things to move fast, the business side must respond fast too (6 min)</t>
+          <t>• What the team is doing to speed up reviews: update on the meeting Dan had with the Risk team, Shawn Street and Trisha (2 min)
+• Ask 1: start working on priorities we can surface in these calls, so we can prioritize requests and guide teams to ours (lots of things come in) (1.5 min)
+• Ask 2: how we show up when entering requests. Example of a really good request; if we want things to move fast, the business side must respond fast too (1.5 min)</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr">
@@ -877,7 +877,7 @@
       </c>
       <c r="K9" s="13" t="inlineStr">
         <is>
-          <t>A few bullets on the meetings. One real example of a strong request.</t>
+          <t>A few bullets on the meetings. One real example of a strong request (could go in a pre-read).</t>
         </is>
       </c>
       <c r="L9" s="13" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="M9" s="13" t="inlineStr">
         <is>
-          <t>Shawn Street is not on the roster.</t>
+          <t>Only 5 minutes: keep the asks tight and take the good-request example as a pre-read. Shawn Street is not on the roster.</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
         <v/>
       </c>
       <c r="D11" s="10" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
@@ -976,9 +976,9 @@
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>• Vision: one place for skills, plugins, connectors and shared context, tagged by role and craft (5 min)
+          <t>• Vision: one place for skills, plugins, connectors and shared context, tagged by role and craft (4 min)
       We do not have the hub yet. Create Hub has started it and is our framework to get kicked off (ties to Design System Agentification)
-• Open discussion: where we see it going, and the value across the org (7 min)</t>
+• Open discussion: where we see it going, and the value across the org (6 min)</t>
         </is>
       </c>
       <c r="H11" s="13" t="inlineStr">
@@ -1078,7 +1078,7 @@
         <v/>
       </c>
       <c r="D13" s="10" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
@@ -1092,10 +1092,10 @@
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>• Other AI priorities the team is working on that I do not know about | Chris McComas, Chris Kostakis (2 min)
+          <t>• Open: other AI priorities the team is working on that I do not know about | Chris McComas, Chris Kostakis (4 min)
 • AI Discoverability | Alex Clemmons, Ethan Hanson (4 min)
 • AI Yields (content audit and enrichment for LLMO) | Markus Sheldon (4 min)
-• Design System Agentification (Create Hub, ties to the hub) | Dave Calleja (4 min)
+• Design System Agentification (Create Hub, ties to the hub) | Dave Calleja (6 min)
 • Salesforce Agentic Harness | Markus Sheldon, Joe Anzalone (4 min)</t>
         </is>
       </c>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="L13" s="13" t="inlineStr">
         <is>
-          <t>Shorten each to 3 min</t>
+          <t>Open ask to 2 min; items to 3 min</t>
         </is>
       </c>
       <c r="M13" s="13" t="inlineStr">
@@ -1202,7 +1202,7 @@
         <v/>
       </c>
       <c r="D15" s="10" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>• Other AI priorities the team is working on that I do not know about | Deana Derocha, Stephen Meyer (2 min)
+          <t>• Open: other AI priorities the team is working on that I do not know about | Deana Derocha, Stephen Meyer (4 min)
 • Client AI Operating Agreement, then discussion: pursue it? who wants to help? value for the group? | Stephen Meyer (5 min)
 • Measurement Framework and Reporting, then the same discussion | Stephen Meyer (5 min)
 • AI Decisioning: AI deciding individual customer journeys in CRM tools (for example Braze, Hightouch) | Barry Latimer (4 min)
@@ -1325,7 +1325,7 @@
         <v/>
       </c>
       <c r="D17" s="10" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
@@ -1339,10 +1339,10 @@
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>• Client &amp; Commercial: tools, initiatives and similar | Mike Monacelli (5 min)
+          <t>• Client &amp; Commercial: tools, initiatives and similar | Mike Monacelli (7 min)
 • AI Commercial guidance: a teaser of where it is going | Alex Willard (3 min)
-• Solutioning: open slot, anything to share? | Tony Toubia (2 min)
-• AI Advisory: open slot, anything to share? | Jason Van Peeren (2 min)
+• Solutioning: open slot, anything to share? | Tony Toubia (3 min)
+• AI Advisory: open slot, anything to share? | Jason Van Peeren (3 min)
 • Romulus: quick walkthrough | Adam Organ (5 min)</t>
         </is>
       </c>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="L17" s="13" t="inlineStr">
         <is>
-          <t>Skip Solutioning and AI Advisory if nothing to share; Mike and Adam to 3 min</t>
+          <t>Skip Solutioning and AI Advisory if nothing to share; Mike to 4 min, Adam to 3 min</t>
         </is>
       </c>
       <c r="M17" s="13" t="inlineStr">
@@ -1390,7 +1390,7 @@
         <v/>
       </c>
       <c r="D18" s="10" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
       <c r="G18" s="13" t="inlineStr">
         <is>
           <t>• Knowledge management teaser: standing up a workforce. Raise hands to see who wants to help (3 min)
-• Open forum: need help? built something cool? Plus the open call: a big problem, something cool, or a team worth showcasing (4 min)
+• Open forum: need help? built something cool? Plus the open call: a big problem, something cool, or a team worth showcasing (6 min)
 • In the news (hot AI things) and announcements (Merkle/dentsu, trainings) (4 min)</t>
         </is>
       </c>
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="C6" s="13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D6" s="13">
         <f>SUM($C$5:C6)</f>
@@ -1665,7 +1665,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Shorten each DBT lightning update from 4 to 3 minutes</t>
+          <t>Shorten the DBT and DDM open asks from 4 to 2 minutes each</t>
         </is>
       </c>
       <c r="C12" s="13" t="n">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="E12" s="13" t="inlineStr">
         <is>
-          <t>A minute per update.</t>
+          <t>Time for surprises from those teams.</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
         </is>
       </c>
       <c r="C13" s="13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D13" s="13">
         <f>SUM($C$5:C13)</f>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>Dan's journey and budget click-down, Risk Review and priorities, the Best practice hub, AI DLC (one of Pete's top priorities), and Design System Agentification (it ties to the hub).</t>
+          <t>Dan's journey and budget click-down, Risk Review and priorities (already only 5 minutes), the Best practice hub, AI DLC (one of Pete's top priorities), and Design System Agentification (it ties to the hub).</t>
         </is>
       </c>
     </row>

</xml_diff>